<commit_message>
Add cards, hero blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (9):
- blocks/cards/_cards.json
- blocks/cards/cards.css
- blocks/hero/_hero.json
- blocks/hero/hero.css
- component-models.json
- tools/importer/import-figma-home.bundle.js
- tools/importer/import-figma-home.js
- tools/importer/reports/ged-pages/figma-home.report.json
- tools/importer/reports/import-figma-home.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-figma-home.report.xlsx
+++ b/tools/importer/reports/import-figma-home.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="82">
   <si>
     <t>_reportFile</t>
   </si>
@@ -25,9 +25,6 @@
     <t>status</t>
   </si>
   <si>
-    <t>stepCount</t>
-  </si>
-  <si>
     <t>template</t>
   </si>
   <si>
@@ -52,9 +49,6 @@
     <t>success</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>home</t>
   </si>
   <si>
@@ -70,7 +64,7 @@
     <t>ged-pages/figma-home.report.json</t>
   </si>
   <si>
-    <t>["accordion (positivus)"]</t>
+    <t>["hero (positivus)","cards (positivus)","accordion (positivus)"]</t>
   </si>
   <si>
     <t>ged-pages/figma-home</t>
@@ -79,7 +73,7 @@
     <t>figma-home</t>
   </si>
   <si>
-    <t>2026-08-18T02:53:26.925Z</t>
+    <t>2026-08-18T04:58:56.753Z</t>
   </si>
   <si>
     <t>Accepting University Search Archive - GED - Other Countries</t>
@@ -651,18 +645,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="41" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="26" customWidth="1"/>
-    <col min="8" max="9" width="50" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -687,360 +680,321 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
       <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="I2" t="s">
+      <c r="B3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
         <v>18</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
         <v>19</v>
       </c>
-      <c r="C3" t="s">
+      <c r="F3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>21</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>22</v>
       </c>
-      <c r="H3" t="s">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>23</v>
       </c>
-      <c r="I3" t="s">
+      <c r="B4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="C4" t="s">
         <v>25</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s">
+      <c r="F4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>28</v>
       </c>
-      <c r="G4" t="s">
+      <c r="B5" t="s">
         <v>29</v>
       </c>
-      <c r="H4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="C5" t="s">
         <v>30</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
         <v>31</v>
       </c>
-      <c r="C5" t="s">
+      <c r="F5" t="s">
         <v>32</v>
       </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>33</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>34</v>
       </c>
-      <c r="H5" t="s">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>35</v>
       </c>
-      <c r="I5" t="s">
+      <c r="B6" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="C6" t="s">
         <v>37</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
         <v>38</v>
       </c>
-      <c r="C6" t="s">
+      <c r="F6" t="s">
         <v>39</v>
       </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>40</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>41</v>
       </c>
-      <c r="H6" t="s">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>42</v>
       </c>
-      <c r="I6" t="s">
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" t="s">
         <v>44</v>
       </c>
-      <c r="B7" t="s">
+      <c r="G7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
         <v>38</v>
       </c>
-      <c r="C7" t="s">
-        <v>45</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" t="s">
-        <v>40</v>
-      </c>
-      <c r="G7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H7" t="s">
-        <v>47</v>
-      </c>
-      <c r="I7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>49</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="F8" t="s">
         <v>50</v>
       </c>
-      <c r="C8" t="s">
+      <c r="G8" t="s">
         <v>51</v>
       </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" t="s">
-        <v>40</v>
-      </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>52</v>
       </c>
-      <c r="H8" t="s">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>53</v>
       </c>
-      <c r="I8" t="s">
+      <c r="B9" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="C9" t="s">
         <v>55</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
         <v>56</v>
       </c>
-      <c r="C9" t="s">
+      <c r="F9" t="s">
         <v>57</v>
       </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>58</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>59</v>
       </c>
-      <c r="H9" t="s">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>60</v>
       </c>
-      <c r="I9" t="s">
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" t="s">
         <v>62</v>
       </c>
-      <c r="B10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="G10" t="s">
         <v>63</v>
       </c>
-      <c r="D10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" t="s">
-        <v>40</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>64</v>
       </c>
-      <c r="H10" t="s">
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>65</v>
       </c>
-      <c r="I10" t="s">
+      <c r="B11" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="C11" t="s">
         <v>67</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
         <v>68</v>
       </c>
-      <c r="C11" t="s">
+      <c r="F11" t="s">
         <v>69</v>
       </c>
-      <c r="D11" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>70</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>71</v>
       </c>
-      <c r="H11" t="s">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>72</v>
       </c>
-      <c r="I11" t="s">
+      <c r="B12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" t="s">
         <v>74</v>
       </c>
-      <c r="B12" t="s">
-        <v>68</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="G12" t="s">
         <v>75</v>
       </c>
-      <c r="D12" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" t="s">
-        <v>70</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>76</v>
       </c>
-      <c r="H12" t="s">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>77</v>
       </c>
-      <c r="I12" t="s">
+      <c r="B13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" t="s">
         <v>79</v>
       </c>
-      <c r="B13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="G13" t="s">
         <v>80</v>
       </c>
-      <c r="D13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" t="s">
-        <v>82</v>
-      </c>
-      <c r="I13" t="s">
-        <v>83</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>